<commit_message>
retire les icônes de copie inertes de la version iPad sans macro
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Racco_D2.xlsx
+++ b/excel/Racco_D2.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="169">
   <si>
     <t>Paramètres</t>
   </si>
@@ -546,9 +546,6 @@
   </si>
   <si>
     <t>+ 30 JOURS</t>
-  </si>
-  <si>
-    <t>⧉</t>
   </si>
   <si>
     <t>+ 65 JOURS</t>
@@ -567,7 +564,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -712,14 +709,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF33190F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color rgb="FF4A4238"/>
       <name val="Consolas"/>
@@ -762,7 +751,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -802,12 +791,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEBE4DC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8907A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -913,7 +896,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1036,40 +1019,37 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1087,7 +1067,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2673,12 +2653,10 @@
       <c r="V28" s="37"/>
       <c r="W28" s="37"/>
       <c r="X28" s="37"/>
-      <c r="Y28" s="38" t="s">
+      <c r="Y28" s="29"/>
+      <c r="Z28" s="29"/>
+      <c r="AA28" s="37" t="s">
         <v>166</v>
-      </c>
-      <c r="Z28" s="38"/>
-      <c r="AA28" s="37" t="s">
-        <v>167</v>
       </c>
       <c r="AB28" s="37"/>
       <c r="AC28" s="37"/>
@@ -2686,10 +2664,8 @@
       <c r="AE28" s="37"/>
       <c r="AF28" s="37"/>
       <c r="AG28" s="37"/>
-      <c r="AH28" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="AI28" s="38"/>
+      <c r="AH28" s="29"/>
+      <c r="AI28" s="29"/>
       <c r="AK28" s="14" t="s">
         <v>71</v>
       </c>
@@ -2704,40 +2680,40 @@
         <v>74</v>
       </c>
       <c r="F29" s="19"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="39"/>
-      <c r="J29" s="39"/>
-      <c r="K29" s="39"/>
-      <c r="L29" s="39"/>
-      <c r="M29" s="39"/>
-      <c r="N29" s="39"/>
-      <c r="O29" s="39"/>
-      <c r="P29" s="39"/>
-      <c r="Q29" s="39"/>
-      <c r="R29" s="40">
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
+      <c r="J29" s="38"/>
+      <c r="K29" s="38"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="38"/>
+      <c r="N29" s="38"/>
+      <c r="O29" s="38"/>
+      <c r="P29" s="38"/>
+      <c r="Q29" s="38"/>
+      <c r="R29" s="39">
         <f>IF(Calcul!$C$945="","—",Calcul!$D$945&amp;" "&amp;Calcul!$C$945)</f>
         <v>0</v>
       </c>
-      <c r="S29" s="40"/>
-      <c r="T29" s="40"/>
-      <c r="U29" s="40"/>
-      <c r="V29" s="40"/>
-      <c r="W29" s="40"/>
-      <c r="X29" s="40"/>
-      <c r="Y29" s="40"/>
-      <c r="Z29" s="40"/>
-      <c r="AA29" s="40">
+      <c r="S29" s="39"/>
+      <c r="T29" s="39"/>
+      <c r="U29" s="39"/>
+      <c r="V29" s="39"/>
+      <c r="W29" s="39"/>
+      <c r="X29" s="39"/>
+      <c r="Y29" s="39"/>
+      <c r="Z29" s="39"/>
+      <c r="AA29" s="39">
         <f>IF(Calcul!$C$946="","—",Calcul!$D$946&amp;" "&amp;Calcul!$C$946)</f>
         <v>0</v>
       </c>
-      <c r="AB29" s="40"/>
-      <c r="AC29" s="40"/>
-      <c r="AD29" s="40"/>
-      <c r="AE29" s="40"/>
-      <c r="AF29" s="40"/>
-      <c r="AG29" s="40"/>
-      <c r="AH29" s="40"/>
-      <c r="AI29" s="40"/>
+      <c r="AB29" s="39"/>
+      <c r="AC29" s="39"/>
+      <c r="AD29" s="39"/>
+      <c r="AE29" s="39"/>
+      <c r="AF29" s="39"/>
+      <c r="AG29" s="39"/>
+      <c r="AH29" s="39"/>
+      <c r="AI29" s="39"/>
       <c r="AK29" s="14" t="s">
         <v>73</v>
       </c>
@@ -2752,43 +2728,43 @@
         <v>76</v>
       </c>
       <c r="F30" s="19"/>
-      <c r="H30" s="41">
+      <c r="H30" s="40">
         <f>IF(ISNUMBER('Racco D2'!$H$29),"Départ · "&amp;CHOOSE(WEEKDAY('Racco D2'!$H$29),"dimanche","lundi","mardi","mercredi","jeudi","vendredi","samedi"),"")</f>
         <v>0</v>
       </c>
-      <c r="I30" s="41"/>
-      <c r="J30" s="41"/>
-      <c r="K30" s="41"/>
-      <c r="L30" s="41"/>
-      <c r="M30" s="41"/>
-      <c r="N30" s="41"/>
-      <c r="O30" s="41"/>
-      <c r="P30" s="41"/>
-      <c r="Q30" s="41"/>
-      <c r="R30" s="42">
+      <c r="I30" s="40"/>
+      <c r="J30" s="40"/>
+      <c r="K30" s="40"/>
+      <c r="L30" s="40"/>
+      <c r="M30" s="40"/>
+      <c r="N30" s="40"/>
+      <c r="O30" s="40"/>
+      <c r="P30" s="40"/>
+      <c r="Q30" s="40"/>
+      <c r="R30" s="41">
         <f>Calcul!$E$945</f>
         <v>0</v>
       </c>
-      <c r="S30" s="42"/>
-      <c r="T30" s="42"/>
-      <c r="U30" s="42"/>
-      <c r="V30" s="42"/>
-      <c r="W30" s="42"/>
-      <c r="X30" s="42"/>
-      <c r="Y30" s="42"/>
-      <c r="Z30" s="42"/>
-      <c r="AA30" s="42">
+      <c r="S30" s="41"/>
+      <c r="T30" s="41"/>
+      <c r="U30" s="41"/>
+      <c r="V30" s="41"/>
+      <c r="W30" s="41"/>
+      <c r="X30" s="41"/>
+      <c r="Y30" s="41"/>
+      <c r="Z30" s="41"/>
+      <c r="AA30" s="41">
         <f>Calcul!$E$946</f>
         <v>0</v>
       </c>
-      <c r="AB30" s="42"/>
-      <c r="AC30" s="42"/>
-      <c r="AD30" s="42"/>
-      <c r="AE30" s="42"/>
-      <c r="AF30" s="42"/>
-      <c r="AG30" s="42"/>
-      <c r="AH30" s="42"/>
-      <c r="AI30" s="42"/>
+      <c r="AB30" s="41"/>
+      <c r="AC30" s="41"/>
+      <c r="AD30" s="41"/>
+      <c r="AE30" s="41"/>
+      <c r="AF30" s="41"/>
+      <c r="AG30" s="41"/>
+      <c r="AH30" s="41"/>
+      <c r="AI30" s="41"/>
       <c r="AK30" s="14" t="s">
         <v>75</v>
       </c>
@@ -2891,36 +2867,36 @@
         <v>82</v>
       </c>
       <c r="F33" s="19"/>
-      <c r="H33" s="43" t="s">
-        <v>168</v>
-      </c>
-      <c r="I33" s="43"/>
-      <c r="J33" s="43"/>
-      <c r="K33" s="43"/>
-      <c r="L33" s="43"/>
-      <c r="M33" s="43"/>
-      <c r="N33" s="43"/>
-      <c r="O33" s="44"/>
-      <c r="P33" s="44"/>
-      <c r="Q33" s="44"/>
-      <c r="R33" s="44"/>
-      <c r="S33" s="44"/>
-      <c r="T33" s="44"/>
-      <c r="U33" s="44"/>
-      <c r="V33" s="44"/>
-      <c r="W33" s="44"/>
-      <c r="X33" s="44"/>
-      <c r="Y33" s="44"/>
-      <c r="Z33" s="44"/>
-      <c r="AA33" s="44"/>
-      <c r="AB33" s="44"/>
-      <c r="AC33" s="44"/>
-      <c r="AD33" s="44"/>
-      <c r="AE33" s="44"/>
-      <c r="AF33" s="44"/>
-      <c r="AG33" s="44"/>
-      <c r="AH33" s="44"/>
-      <c r="AI33" s="44"/>
+      <c r="H33" s="42" t="s">
+        <v>167</v>
+      </c>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="43"/>
+      <c r="P33" s="43"/>
+      <c r="Q33" s="43"/>
+      <c r="R33" s="43"/>
+      <c r="S33" s="43"/>
+      <c r="T33" s="43"/>
+      <c r="U33" s="43"/>
+      <c r="V33" s="43"/>
+      <c r="W33" s="43"/>
+      <c r="X33" s="43"/>
+      <c r="Y33" s="43"/>
+      <c r="Z33" s="43"/>
+      <c r="AA33" s="43"/>
+      <c r="AB33" s="43"/>
+      <c r="AC33" s="43"/>
+      <c r="AD33" s="43"/>
+      <c r="AE33" s="43"/>
+      <c r="AF33" s="43"/>
+      <c r="AG33" s="43"/>
+      <c r="AH33" s="43"/>
+      <c r="AI33" s="43"/>
       <c r="AK33" s="14" t="s">
         <v>81</v>
       </c>
@@ -2949,12 +2925,10 @@
       <c r="Q34" s="37"/>
       <c r="R34" s="37"/>
       <c r="S34" s="37"/>
-      <c r="T34" s="38" t="s">
+      <c r="T34" s="29"/>
+      <c r="U34" s="29"/>
+      <c r="V34" s="37" t="s">
         <v>166</v>
-      </c>
-      <c r="U34" s="38"/>
-      <c r="V34" s="37" t="s">
-        <v>167</v>
       </c>
       <c r="W34" s="37"/>
       <c r="X34" s="37"/>
@@ -2967,10 +2941,8 @@
       <c r="AE34" s="37"/>
       <c r="AF34" s="37"/>
       <c r="AG34" s="37"/>
-      <c r="AH34" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="AI34" s="38"/>
+      <c r="AH34" s="29"/>
+      <c r="AI34" s="29"/>
       <c r="AK34" s="14" t="s">
         <v>84</v>
       </c>
@@ -2985,46 +2957,46 @@
         <v>87</v>
       </c>
       <c r="F35" s="19"/>
-      <c r="H35" s="40">
+      <c r="H35" s="39">
         <f>IF(Calcul!$C$945="","—",Calcul!$D$945&amp;" "&amp;Calcul!$C$945)</f>
         <v>0</v>
       </c>
-      <c r="I35" s="40"/>
-      <c r="J35" s="40"/>
-      <c r="K35" s="40"/>
-      <c r="L35" s="40"/>
-      <c r="M35" s="40"/>
-      <c r="N35" s="40"/>
-      <c r="O35" s="40"/>
-      <c r="P35" s="40"/>
-      <c r="Q35" s="40"/>
-      <c r="R35" s="45">
+      <c r="I35" s="39"/>
+      <c r="J35" s="39"/>
+      <c r="K35" s="39"/>
+      <c r="L35" s="39"/>
+      <c r="M35" s="39"/>
+      <c r="N35" s="39"/>
+      <c r="O35" s="39"/>
+      <c r="P35" s="39"/>
+      <c r="Q35" s="39"/>
+      <c r="R35" s="44">
         <f>Calcul!$E$945</f>
         <v>0</v>
       </c>
-      <c r="S35" s="45"/>
-      <c r="T35" s="45"/>
-      <c r="U35" s="45"/>
-      <c r="V35" s="40">
+      <c r="S35" s="44"/>
+      <c r="T35" s="44"/>
+      <c r="U35" s="44"/>
+      <c r="V35" s="39">
         <f>IF(Calcul!$C$946="","—",Calcul!$D$946&amp;" "&amp;Calcul!$C$946)</f>
         <v>0</v>
       </c>
-      <c r="W35" s="40"/>
-      <c r="X35" s="40"/>
-      <c r="Y35" s="40"/>
-      <c r="Z35" s="40"/>
-      <c r="AA35" s="40"/>
-      <c r="AB35" s="40"/>
-      <c r="AC35" s="40"/>
-      <c r="AD35" s="40"/>
-      <c r="AE35" s="40"/>
-      <c r="AF35" s="45">
+      <c r="W35" s="39"/>
+      <c r="X35" s="39"/>
+      <c r="Y35" s="39"/>
+      <c r="Z35" s="39"/>
+      <c r="AA35" s="39"/>
+      <c r="AB35" s="39"/>
+      <c r="AC35" s="39"/>
+      <c r="AD35" s="39"/>
+      <c r="AE35" s="39"/>
+      <c r="AF35" s="44">
         <f>Calcul!$E$946</f>
         <v>0</v>
       </c>
-      <c r="AG35" s="45"/>
-      <c r="AH35" s="45"/>
-      <c r="AI35" s="45"/>
+      <c r="AG35" s="44"/>
+      <c r="AH35" s="44"/>
+      <c r="AI35" s="44"/>
       <c r="AK35" s="14" t="s">
         <v>86</v>
       </c>
@@ -3037,34 +3009,34 @@
         <v>146</v>
       </c>
       <c r="F36" s="29"/>
-      <c r="H36" s="44"/>
-      <c r="I36" s="44"/>
-      <c r="J36" s="44"/>
-      <c r="K36" s="44"/>
-      <c r="L36" s="44"/>
-      <c r="M36" s="44"/>
-      <c r="N36" s="44"/>
-      <c r="O36" s="44"/>
-      <c r="P36" s="44"/>
-      <c r="Q36" s="44"/>
-      <c r="R36" s="44"/>
-      <c r="S36" s="44"/>
-      <c r="T36" s="44"/>
-      <c r="U36" s="44"/>
-      <c r="V36" s="44"/>
-      <c r="W36" s="44"/>
-      <c r="X36" s="44"/>
-      <c r="Y36" s="44"/>
-      <c r="Z36" s="44"/>
-      <c r="AA36" s="44"/>
-      <c r="AB36" s="44"/>
-      <c r="AC36" s="44"/>
-      <c r="AD36" s="44"/>
-      <c r="AE36" s="44"/>
-      <c r="AF36" s="44"/>
-      <c r="AG36" s="44"/>
-      <c r="AH36" s="44"/>
-      <c r="AI36" s="44"/>
+      <c r="H36" s="43"/>
+      <c r="I36" s="43"/>
+      <c r="J36" s="43"/>
+      <c r="K36" s="43"/>
+      <c r="L36" s="43"/>
+      <c r="M36" s="43"/>
+      <c r="N36" s="43"/>
+      <c r="O36" s="43"/>
+      <c r="P36" s="43"/>
+      <c r="Q36" s="43"/>
+      <c r="R36" s="43"/>
+      <c r="S36" s="43"/>
+      <c r="T36" s="43"/>
+      <c r="U36" s="43"/>
+      <c r="V36" s="43"/>
+      <c r="W36" s="43"/>
+      <c r="X36" s="43"/>
+      <c r="Y36" s="43"/>
+      <c r="Z36" s="43"/>
+      <c r="AA36" s="43"/>
+      <c r="AB36" s="43"/>
+      <c r="AC36" s="43"/>
+      <c r="AD36" s="43"/>
+      <c r="AE36" s="43"/>
+      <c r="AF36" s="43"/>
+      <c r="AG36" s="43"/>
+      <c r="AH36" s="43"/>
+      <c r="AI36" s="43"/>
       <c r="AK36" s="14" t="s">
         <v>146</v>
       </c>
@@ -3079,38 +3051,36 @@
         <v>89</v>
       </c>
       <c r="F37" s="19"/>
-      <c r="H37" s="46" t="s">
-        <v>169</v>
-      </c>
-      <c r="I37" s="46"/>
-      <c r="J37" s="46"/>
-      <c r="K37" s="46"/>
-      <c r="L37" s="46"/>
-      <c r="M37" s="46"/>
-      <c r="N37" s="46"/>
-      <c r="O37" s="46"/>
-      <c r="P37" s="46"/>
-      <c r="Q37" s="46"/>
-      <c r="R37" s="46"/>
-      <c r="S37" s="46"/>
-      <c r="T37" s="46"/>
-      <c r="U37" s="46"/>
-      <c r="V37" s="46"/>
-      <c r="W37" s="46"/>
-      <c r="X37" s="46"/>
-      <c r="Y37" s="46"/>
-      <c r="Z37" s="46"/>
-      <c r="AA37" s="46"/>
-      <c r="AB37" s="46"/>
-      <c r="AC37" s="46"/>
-      <c r="AD37" s="46"/>
-      <c r="AE37" s="46"/>
-      <c r="AF37" s="46"/>
-      <c r="AG37" s="46"/>
-      <c r="AH37" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="AI37" s="38"/>
+      <c r="H37" s="45" t="s">
+        <v>168</v>
+      </c>
+      <c r="I37" s="45"/>
+      <c r="J37" s="45"/>
+      <c r="K37" s="45"/>
+      <c r="L37" s="45"/>
+      <c r="M37" s="45"/>
+      <c r="N37" s="45"/>
+      <c r="O37" s="45"/>
+      <c r="P37" s="45"/>
+      <c r="Q37" s="45"/>
+      <c r="R37" s="45"/>
+      <c r="S37" s="45"/>
+      <c r="T37" s="45"/>
+      <c r="U37" s="45"/>
+      <c r="V37" s="45"/>
+      <c r="W37" s="45"/>
+      <c r="X37" s="45"/>
+      <c r="Y37" s="45"/>
+      <c r="Z37" s="45"/>
+      <c r="AA37" s="45"/>
+      <c r="AB37" s="45"/>
+      <c r="AC37" s="45"/>
+      <c r="AD37" s="45"/>
+      <c r="AE37" s="45"/>
+      <c r="AF37" s="45"/>
+      <c r="AG37" s="45"/>
+      <c r="AH37" s="29"/>
+      <c r="AI37" s="29"/>
       <c r="AK37" s="14" t="s">
         <v>88</v>
       </c>
@@ -3125,37 +3095,37 @@
         <v>92</v>
       </c>
       <c r="F38" s="19"/>
-      <c r="H38" s="47">
+      <c r="H38" s="46">
         <f>MID(Calcul!$B$82,1,5)&amp;" "&amp;MID(Calcul!$B$82,6,5)&amp;" "&amp;MID(Calcul!$B$82,11,5)&amp;" "&amp;MID(Calcul!$B$82,16,5)&amp;" "&amp;MID(Calcul!$B$82,21,5)</f>
         <v>0</v>
       </c>
-      <c r="I38" s="47"/>
-      <c r="J38" s="47"/>
-      <c r="K38" s="47"/>
-      <c r="L38" s="47"/>
-      <c r="M38" s="47"/>
-      <c r="N38" s="47"/>
-      <c r="O38" s="47"/>
-      <c r="P38" s="47"/>
-      <c r="Q38" s="47"/>
-      <c r="R38" s="47"/>
-      <c r="S38" s="47"/>
-      <c r="T38" s="47"/>
-      <c r="U38" s="47"/>
-      <c r="V38" s="47"/>
-      <c r="W38" s="47"/>
-      <c r="X38" s="47"/>
-      <c r="Y38" s="47"/>
-      <c r="Z38" s="47"/>
-      <c r="AA38" s="47"/>
-      <c r="AB38" s="47"/>
-      <c r="AC38" s="47"/>
-      <c r="AD38" s="47"/>
-      <c r="AE38" s="47"/>
-      <c r="AF38" s="47"/>
-      <c r="AG38" s="47"/>
-      <c r="AH38" s="47"/>
-      <c r="AI38" s="47"/>
+      <c r="I38" s="46"/>
+      <c r="J38" s="46"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="46"/>
+      <c r="Q38" s="46"/>
+      <c r="R38" s="46"/>
+      <c r="S38" s="46"/>
+      <c r="T38" s="46"/>
+      <c r="U38" s="46"/>
+      <c r="V38" s="46"/>
+      <c r="W38" s="46"/>
+      <c r="X38" s="46"/>
+      <c r="Y38" s="46"/>
+      <c r="Z38" s="46"/>
+      <c r="AA38" s="46"/>
+      <c r="AB38" s="46"/>
+      <c r="AC38" s="46"/>
+      <c r="AD38" s="46"/>
+      <c r="AE38" s="46"/>
+      <c r="AF38" s="46"/>
+      <c r="AG38" s="46"/>
+      <c r="AH38" s="46"/>
+      <c r="AI38" s="46"/>
       <c r="AK38" s="14" t="s">
         <v>91</v>
       </c>
@@ -3170,34 +3140,34 @@
         <v>94</v>
       </c>
       <c r="F39" s="19"/>
-      <c r="H39" s="44"/>
-      <c r="I39" s="44"/>
-      <c r="J39" s="44"/>
-      <c r="K39" s="44"/>
-      <c r="L39" s="44"/>
-      <c r="M39" s="44"/>
-      <c r="N39" s="44"/>
-      <c r="O39" s="44"/>
-      <c r="P39" s="44"/>
-      <c r="Q39" s="44"/>
-      <c r="R39" s="44"/>
-      <c r="S39" s="44"/>
-      <c r="T39" s="44"/>
-      <c r="U39" s="44"/>
-      <c r="V39" s="44"/>
-      <c r="W39" s="44"/>
-      <c r="X39" s="44"/>
-      <c r="Y39" s="44"/>
-      <c r="Z39" s="44"/>
-      <c r="AA39" s="44"/>
-      <c r="AB39" s="44"/>
-      <c r="AC39" s="44"/>
-      <c r="AD39" s="44"/>
-      <c r="AE39" s="44"/>
-      <c r="AF39" s="44"/>
-      <c r="AG39" s="44"/>
-      <c r="AH39" s="44"/>
-      <c r="AI39" s="44"/>
+      <c r="H39" s="43"/>
+      <c r="I39" s="43"/>
+      <c r="J39" s="43"/>
+      <c r="K39" s="43"/>
+      <c r="L39" s="43"/>
+      <c r="M39" s="43"/>
+      <c r="N39" s="43"/>
+      <c r="O39" s="43"/>
+      <c r="P39" s="43"/>
+      <c r="Q39" s="43"/>
+      <c r="R39" s="43"/>
+      <c r="S39" s="43"/>
+      <c r="T39" s="43"/>
+      <c r="U39" s="43"/>
+      <c r="V39" s="43"/>
+      <c r="W39" s="43"/>
+      <c r="X39" s="43"/>
+      <c r="Y39" s="43"/>
+      <c r="Z39" s="43"/>
+      <c r="AA39" s="43"/>
+      <c r="AB39" s="43"/>
+      <c r="AC39" s="43"/>
+      <c r="AD39" s="43"/>
+      <c r="AE39" s="43"/>
+      <c r="AF39" s="43"/>
+      <c r="AG39" s="43"/>
+      <c r="AH39" s="43"/>
+      <c r="AI39" s="43"/>
       <c r="AK39" s="14" t="s">
         <v>93</v>
       </c>
@@ -3216,48 +3186,44 @@
       <c r="F40" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="H40" s="48" t="s">
+      <c r="H40" s="47" t="s">
         <v>127</v>
       </c>
-      <c r="I40" s="48"/>
-      <c r="J40" s="48"/>
-      <c r="K40" s="49">
+      <c r="I40" s="47"/>
+      <c r="J40" s="47"/>
+      <c r="K40" s="48">
         <f>MID(Calcul!$B$329,1,5)&amp;" "&amp;MID(Calcul!$B$329,6,5)&amp;" "&amp;MID(Calcul!$B$329,11,5)</f>
         <v>0</v>
       </c>
-      <c r="L40" s="49"/>
-      <c r="M40" s="49"/>
-      <c r="N40" s="49"/>
-      <c r="O40" s="49"/>
-      <c r="P40" s="49"/>
-      <c r="Q40" s="49"/>
-      <c r="R40" s="49"/>
-      <c r="S40" s="49"/>
-      <c r="T40" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="U40" s="38"/>
-      <c r="V40" s="48" t="s">
+      <c r="L40" s="48"/>
+      <c r="M40" s="48"/>
+      <c r="N40" s="48"/>
+      <c r="O40" s="48"/>
+      <c r="P40" s="48"/>
+      <c r="Q40" s="48"/>
+      <c r="R40" s="48"/>
+      <c r="S40" s="48"/>
+      <c r="T40" s="29"/>
+      <c r="U40" s="29"/>
+      <c r="V40" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="W40" s="48"/>
-      <c r="X40" s="48"/>
-      <c r="Y40" s="49">
+      <c r="W40" s="47"/>
+      <c r="X40" s="47"/>
+      <c r="Y40" s="48">
         <f>MID(Calcul!$B$637,1,5)&amp;" "&amp;MID(Calcul!$B$637,6,5)&amp;" "&amp;MID(Calcul!$B$637,11,5)&amp;" "&amp;MID(Calcul!$B$637,16,5)</f>
         <v>0</v>
       </c>
-      <c r="Z40" s="49"/>
-      <c r="AA40" s="49"/>
-      <c r="AB40" s="49"/>
-      <c r="AC40" s="49"/>
-      <c r="AD40" s="49"/>
-      <c r="AE40" s="49"/>
-      <c r="AF40" s="49"/>
-      <c r="AG40" s="49"/>
-      <c r="AH40" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="AI40" s="38"/>
+      <c r="Z40" s="48"/>
+      <c r="AA40" s="48"/>
+      <c r="AB40" s="48"/>
+      <c r="AC40" s="48"/>
+      <c r="AD40" s="48"/>
+      <c r="AE40" s="48"/>
+      <c r="AF40" s="48"/>
+      <c r="AG40" s="48"/>
+      <c r="AH40" s="29"/>
+      <c r="AI40" s="29"/>
       <c r="AK40" s="14" t="s">
         <v>95</v>
       </c>
@@ -3272,34 +3238,34 @@
         <v>98</v>
       </c>
       <c r="F41" s="19"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="44"/>
-      <c r="J41" s="44"/>
-      <c r="K41" s="44"/>
-      <c r="L41" s="44"/>
-      <c r="M41" s="44"/>
-      <c r="N41" s="44"/>
-      <c r="O41" s="44"/>
-      <c r="P41" s="44"/>
-      <c r="Q41" s="44"/>
-      <c r="R41" s="44"/>
-      <c r="S41" s="44"/>
-      <c r="T41" s="44"/>
-      <c r="U41" s="44"/>
-      <c r="V41" s="44"/>
-      <c r="W41" s="44"/>
-      <c r="X41" s="44"/>
-      <c r="Y41" s="44"/>
-      <c r="Z41" s="44"/>
-      <c r="AA41" s="44"/>
-      <c r="AB41" s="44"/>
-      <c r="AC41" s="44"/>
-      <c r="AD41" s="44"/>
-      <c r="AE41" s="44"/>
-      <c r="AF41" s="44"/>
-      <c r="AG41" s="44"/>
-      <c r="AH41" s="44"/>
-      <c r="AI41" s="44"/>
+      <c r="H41" s="43"/>
+      <c r="I41" s="43"/>
+      <c r="J41" s="43"/>
+      <c r="K41" s="43"/>
+      <c r="L41" s="43"/>
+      <c r="M41" s="43"/>
+      <c r="N41" s="43"/>
+      <c r="O41" s="43"/>
+      <c r="P41" s="43"/>
+      <c r="Q41" s="43"/>
+      <c r="R41" s="43"/>
+      <c r="S41" s="43"/>
+      <c r="T41" s="43"/>
+      <c r="U41" s="43"/>
+      <c r="V41" s="43"/>
+      <c r="W41" s="43"/>
+      <c r="X41" s="43"/>
+      <c r="Y41" s="43"/>
+      <c r="Z41" s="43"/>
+      <c r="AA41" s="43"/>
+      <c r="AB41" s="43"/>
+      <c r="AC41" s="43"/>
+      <c r="AD41" s="43"/>
+      <c r="AE41" s="43"/>
+      <c r="AF41" s="43"/>
+      <c r="AG41" s="43"/>
+      <c r="AH41" s="43"/>
+      <c r="AI41" s="43"/>
       <c r="AK41" s="14" t="s">
         <v>97</v>
       </c>
@@ -3314,48 +3280,44 @@
         <v>100</v>
       </c>
       <c r="F42" s="19"/>
-      <c r="H42" s="48" t="s">
+      <c r="H42" s="47" t="s">
         <v>140</v>
       </c>
-      <c r="I42" s="48"/>
-      <c r="J42" s="48"/>
-      <c r="K42" s="49">
+      <c r="I42" s="47"/>
+      <c r="J42" s="47"/>
+      <c r="K42" s="48">
         <f>MID(Calcul!$B$790,1,5)&amp;" "&amp;MID(Calcul!$B$790,6,5)</f>
         <v>0</v>
       </c>
-      <c r="L42" s="49"/>
-      <c r="M42" s="49"/>
-      <c r="N42" s="49"/>
-      <c r="O42" s="49"/>
-      <c r="P42" s="49"/>
-      <c r="Q42" s="49"/>
-      <c r="R42" s="49"/>
-      <c r="S42" s="49"/>
-      <c r="T42" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="U42" s="38"/>
-      <c r="V42" s="48" t="s">
+      <c r="L42" s="48"/>
+      <c r="M42" s="48"/>
+      <c r="N42" s="48"/>
+      <c r="O42" s="48"/>
+      <c r="P42" s="48"/>
+      <c r="Q42" s="48"/>
+      <c r="R42" s="48"/>
+      <c r="S42" s="48"/>
+      <c r="T42" s="29"/>
+      <c r="U42" s="29"/>
+      <c r="V42" s="47" t="s">
         <v>141</v>
       </c>
-      <c r="W42" s="48"/>
-      <c r="X42" s="48"/>
-      <c r="Y42" s="49">
+      <c r="W42" s="47"/>
+      <c r="X42" s="47"/>
+      <c r="Y42" s="48">
         <f>MID(Calcul!$B$943,1,5)&amp;" "&amp;MID(Calcul!$B$943,6,5)</f>
         <v>0</v>
       </c>
-      <c r="Z42" s="49"/>
-      <c r="AA42" s="49"/>
-      <c r="AB42" s="49"/>
-      <c r="AC42" s="49"/>
-      <c r="AD42" s="49"/>
-      <c r="AE42" s="49"/>
-      <c r="AF42" s="49"/>
-      <c r="AG42" s="49"/>
-      <c r="AH42" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="AI42" s="38"/>
+      <c r="Z42" s="48"/>
+      <c r="AA42" s="48"/>
+      <c r="AB42" s="48"/>
+      <c r="AC42" s="48"/>
+      <c r="AD42" s="48"/>
+      <c r="AE42" s="48"/>
+      <c r="AF42" s="48"/>
+      <c r="AG42" s="48"/>
+      <c r="AH42" s="29"/>
+      <c r="AI42" s="29"/>
       <c r="AK42" s="14" t="s">
         <v>99</v>
       </c>
@@ -3370,34 +3332,34 @@
         <v>102</v>
       </c>
       <c r="F43" s="19"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="44"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="44"/>
-      <c r="L43" s="44"/>
-      <c r="M43" s="44"/>
-      <c r="N43" s="44"/>
-      <c r="O43" s="44"/>
-      <c r="P43" s="44"/>
-      <c r="Q43" s="44"/>
-      <c r="R43" s="44"/>
-      <c r="S43" s="44"/>
-      <c r="T43" s="44"/>
-      <c r="U43" s="44"/>
-      <c r="V43" s="44"/>
-      <c r="W43" s="44"/>
-      <c r="X43" s="44"/>
-      <c r="Y43" s="44"/>
-      <c r="Z43" s="44"/>
-      <c r="AA43" s="44"/>
-      <c r="AB43" s="44"/>
-      <c r="AC43" s="44"/>
-      <c r="AD43" s="44"/>
-      <c r="AE43" s="44"/>
-      <c r="AF43" s="44"/>
-      <c r="AG43" s="44"/>
-      <c r="AH43" s="44"/>
-      <c r="AI43" s="44"/>
+      <c r="H43" s="43"/>
+      <c r="I43" s="43"/>
+      <c r="J43" s="43"/>
+      <c r="K43" s="43"/>
+      <c r="L43" s="43"/>
+      <c r="M43" s="43"/>
+      <c r="N43" s="43"/>
+      <c r="O43" s="43"/>
+      <c r="P43" s="43"/>
+      <c r="Q43" s="43"/>
+      <c r="R43" s="43"/>
+      <c r="S43" s="43"/>
+      <c r="T43" s="43"/>
+      <c r="U43" s="43"/>
+      <c r="V43" s="43"/>
+      <c r="W43" s="43"/>
+      <c r="X43" s="43"/>
+      <c r="Y43" s="43"/>
+      <c r="Z43" s="43"/>
+      <c r="AA43" s="43"/>
+      <c r="AB43" s="43"/>
+      <c r="AC43" s="43"/>
+      <c r="AD43" s="43"/>
+      <c r="AE43" s="43"/>
+      <c r="AF43" s="43"/>
+      <c r="AG43" s="43"/>
+      <c r="AH43" s="43"/>
+      <c r="AI43" s="43"/>
       <c r="AK43" s="14" t="s">
         <v>101</v>
       </c>
@@ -3408,34 +3370,34 @@
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
-      <c r="H44" s="44"/>
-      <c r="I44" s="44"/>
-      <c r="J44" s="44"/>
-      <c r="K44" s="44"/>
-      <c r="L44" s="44"/>
-      <c r="M44" s="44"/>
-      <c r="N44" s="44"/>
-      <c r="O44" s="44"/>
-      <c r="P44" s="44"/>
-      <c r="Q44" s="44"/>
-      <c r="R44" s="44"/>
-      <c r="S44" s="44"/>
-      <c r="T44" s="44"/>
-      <c r="U44" s="44"/>
-      <c r="V44" s="44"/>
-      <c r="W44" s="44"/>
-      <c r="X44" s="44"/>
-      <c r="Y44" s="44"/>
-      <c r="Z44" s="44"/>
-      <c r="AA44" s="44"/>
-      <c r="AB44" s="44"/>
-      <c r="AC44" s="44"/>
-      <c r="AD44" s="44"/>
-      <c r="AE44" s="44"/>
-      <c r="AF44" s="44"/>
-      <c r="AG44" s="44"/>
-      <c r="AH44" s="44"/>
-      <c r="AI44" s="44"/>
+      <c r="H44" s="43"/>
+      <c r="I44" s="43"/>
+      <c r="J44" s="43"/>
+      <c r="K44" s="43"/>
+      <c r="L44" s="43"/>
+      <c r="M44" s="43"/>
+      <c r="N44" s="43"/>
+      <c r="O44" s="43"/>
+      <c r="P44" s="43"/>
+      <c r="Q44" s="43"/>
+      <c r="R44" s="43"/>
+      <c r="S44" s="43"/>
+      <c r="T44" s="43"/>
+      <c r="U44" s="43"/>
+      <c r="V44" s="43"/>
+      <c r="W44" s="43"/>
+      <c r="X44" s="43"/>
+      <c r="Y44" s="43"/>
+      <c r="Z44" s="43"/>
+      <c r="AA44" s="43"/>
+      <c r="AB44" s="43"/>
+      <c r="AC44" s="43"/>
+      <c r="AD44" s="43"/>
+      <c r="AE44" s="43"/>
+      <c r="AF44" s="43"/>
+      <c r="AG44" s="43"/>
+      <c r="AH44" s="43"/>
+      <c r="AI44" s="43"/>
       <c r="AK44" s="14"/>
     </row>
     <row r="45" spans="2:37" ht="18" customHeight="1">
@@ -3444,34 +3406,34 @@
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
-      <c r="H45" s="44"/>
-      <c r="I45" s="44"/>
-      <c r="J45" s="44"/>
-      <c r="K45" s="44"/>
-      <c r="L45" s="44"/>
-      <c r="M45" s="44"/>
-      <c r="N45" s="44"/>
-      <c r="O45" s="44"/>
-      <c r="P45" s="44"/>
-      <c r="Q45" s="44"/>
-      <c r="R45" s="44"/>
-      <c r="S45" s="44"/>
-      <c r="T45" s="44"/>
-      <c r="U45" s="44"/>
-      <c r="V45" s="44"/>
-      <c r="W45" s="44"/>
-      <c r="X45" s="44"/>
-      <c r="Y45" s="44"/>
-      <c r="Z45" s="44"/>
-      <c r="AA45" s="44"/>
-      <c r="AB45" s="44"/>
-      <c r="AC45" s="44"/>
-      <c r="AD45" s="44"/>
-      <c r="AE45" s="44"/>
-      <c r="AF45" s="44"/>
-      <c r="AG45" s="44"/>
-      <c r="AH45" s="44"/>
-      <c r="AI45" s="44"/>
+      <c r="H45" s="43"/>
+      <c r="I45" s="43"/>
+      <c r="J45" s="43"/>
+      <c r="K45" s="43"/>
+      <c r="L45" s="43"/>
+      <c r="M45" s="43"/>
+      <c r="N45" s="43"/>
+      <c r="O45" s="43"/>
+      <c r="P45" s="43"/>
+      <c r="Q45" s="43"/>
+      <c r="R45" s="43"/>
+      <c r="S45" s="43"/>
+      <c r="T45" s="43"/>
+      <c r="U45" s="43"/>
+      <c r="V45" s="43"/>
+      <c r="W45" s="43"/>
+      <c r="X45" s="43"/>
+      <c r="Y45" s="43"/>
+      <c r="Z45" s="43"/>
+      <c r="AA45" s="43"/>
+      <c r="AB45" s="43"/>
+      <c r="AC45" s="43"/>
+      <c r="AD45" s="43"/>
+      <c r="AE45" s="43"/>
+      <c r="AF45" s="43"/>
+      <c r="AG45" s="43"/>
+      <c r="AH45" s="43"/>
+      <c r="AI45" s="43"/>
       <c r="AK45" s="14"/>
     </row>
     <row r="46" spans="2:37" ht="18" customHeight="1">
@@ -3480,34 +3442,34 @@
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
-      <c r="H46" s="44"/>
-      <c r="I46" s="44"/>
-      <c r="J46" s="44"/>
-      <c r="K46" s="44"/>
-      <c r="L46" s="44"/>
-      <c r="M46" s="44"/>
-      <c r="N46" s="44"/>
-      <c r="O46" s="44"/>
-      <c r="P46" s="44"/>
-      <c r="Q46" s="44"/>
-      <c r="R46" s="44"/>
-      <c r="S46" s="44"/>
-      <c r="T46" s="44"/>
-      <c r="U46" s="44"/>
-      <c r="V46" s="44"/>
-      <c r="W46" s="44"/>
-      <c r="X46" s="44"/>
-      <c r="Y46" s="44"/>
-      <c r="Z46" s="44"/>
-      <c r="AA46" s="44"/>
-      <c r="AB46" s="44"/>
-      <c r="AC46" s="44"/>
-      <c r="AD46" s="44"/>
-      <c r="AE46" s="44"/>
-      <c r="AF46" s="44"/>
-      <c r="AG46" s="44"/>
-      <c r="AH46" s="44"/>
-      <c r="AI46" s="44"/>
+      <c r="H46" s="43"/>
+      <c r="I46" s="43"/>
+      <c r="J46" s="43"/>
+      <c r="K46" s="43"/>
+      <c r="L46" s="43"/>
+      <c r="M46" s="43"/>
+      <c r="N46" s="43"/>
+      <c r="O46" s="43"/>
+      <c r="P46" s="43"/>
+      <c r="Q46" s="43"/>
+      <c r="R46" s="43"/>
+      <c r="S46" s="43"/>
+      <c r="T46" s="43"/>
+      <c r="U46" s="43"/>
+      <c r="V46" s="43"/>
+      <c r="W46" s="43"/>
+      <c r="X46" s="43"/>
+      <c r="Y46" s="43"/>
+      <c r="Z46" s="43"/>
+      <c r="AA46" s="43"/>
+      <c r="AB46" s="43"/>
+      <c r="AC46" s="43"/>
+      <c r="AD46" s="43"/>
+      <c r="AE46" s="43"/>
+      <c r="AF46" s="43"/>
+      <c r="AG46" s="43"/>
+      <c r="AH46" s="43"/>
+      <c r="AI46" s="43"/>
       <c r="AK46" s="14"/>
     </row>
     <row r="47" spans="2:37" ht="18" customHeight="1">
@@ -3841,46 +3803,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="50" t="s">
+      <c r="C1" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="D1" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="E1" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="50" t="s">
+      <c r="F1" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="50" t="s">
+      <c r="G1" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="50" t="s">
+      <c r="H1" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="50" t="s">
+      <c r="I1" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="50" t="s">
+      <c r="J1" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="50" t="s">
+      <c r="K1" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="50" t="s">
+      <c r="L1" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="M1" s="50" t="s">
+      <c r="M1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="N1" s="50" t="s">
+      <c r="N1" s="49" t="s">
         <v>20</v>
       </c>
     </row>
@@ -5543,58 +5505,58 @@
       </c>
     </row>
     <row r="42" spans="1:18">
-      <c r="A42" s="50" t="s">
+      <c r="A42" s="49" t="s">
         <v>103</v>
       </c>
-      <c r="B42" s="50" t="s">
+      <c r="B42" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="50" t="s">
+      <c r="C42" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="50" t="s">
+      <c r="D42" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="50" t="s">
+      <c r="E42" s="49" t="s">
         <v>104</v>
       </c>
-      <c r="F42" s="50" t="s">
+      <c r="F42" s="49" t="s">
         <v>105</v>
       </c>
-      <c r="G42" s="50" t="s">
+      <c r="G42" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="H42" s="50" t="s">
+      <c r="H42" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="I42" s="50" t="s">
+      <c r="I42" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="J42" s="50" t="s">
+      <c r="J42" s="49" t="s">
         <v>108</v>
       </c>
-      <c r="K42" s="50" t="s">
+      <c r="K42" s="49" t="s">
         <v>109</v>
       </c>
-      <c r="L42" s="50" t="s">
+      <c r="L42" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="M42" s="50" t="s">
+      <c r="M42" s="49" t="s">
         <v>110</v>
       </c>
-      <c r="N42" s="50" t="s">
+      <c r="N42" s="49" t="s">
         <v>111</v>
       </c>
-      <c r="O42" s="50" t="s">
+      <c r="O42" s="49" t="s">
         <v>112</v>
       </c>
-      <c r="P42" s="50" t="s">
+      <c r="P42" s="49" t="s">
         <v>113</v>
       </c>
-      <c r="Q42" s="50" t="s">
+      <c r="Q42" s="49" t="s">
         <v>114</v>
       </c>
-      <c r="R42" s="50" t="s">
+      <c r="R42" s="49" t="s">
         <v>115</v>
       </c>
     </row>
@@ -6047,7 +6009,7 @@
       </c>
     </row>
     <row r="57" spans="1:18">
-      <c r="A57" s="50" t="s">
+      <c r="A57" s="49" t="s">
         <v>121</v>
       </c>
     </row>
@@ -6354,7 +6316,7 @@
       </c>
     </row>
     <row r="85" spans="1:3">
-      <c r="A85" s="50" t="s">
+      <c r="A85" s="49" t="s">
         <v>127</v>
       </c>
     </row>
@@ -8790,7 +8752,7 @@
       </c>
     </row>
     <row r="331" spans="1:3">
-      <c r="A331" s="50" t="s">
+      <c r="A331" s="49" t="s">
         <v>137</v>
       </c>
     </row>
@@ -11844,7 +11806,7 @@
       </c>
     </row>
     <row r="639" spans="1:3">
-      <c r="A639" s="50" t="s">
+      <c r="A639" s="49" t="s">
         <v>140</v>
       </c>
     </row>
@@ -13353,7 +13315,7 @@
       </c>
     </row>
     <row r="792" spans="1:3">
-      <c r="A792" s="50" t="s">
+      <c r="A792" s="49" t="s">
         <v>141</v>
       </c>
     </row>
@@ -14918,1244 +14880,1244 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="51" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="52" t="s">
+      <c r="A1" s="50" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="51" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="54">
+      <c r="B2" s="53">
         <v>30</v>
       </c>
-      <c r="D2" s="55" t="s">
+      <c r="D2" s="54" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="54">
+      <c r="B3" s="53">
         <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="50" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="B6" s="56">
+      <c r="B6" s="55">
         <v>45292</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="B7" s="56">
+      <c r="B7" s="55">
         <v>45383</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="B8" s="56">
+      <c r="B8" s="55">
         <v>45413</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="B9" s="56">
+      <c r="B9" s="55">
         <v>45420</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="B10" s="56">
+      <c r="B10" s="55">
         <v>45421</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="B11" s="56">
+      <c r="B11" s="55">
         <v>45432</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="B12" s="56">
+      <c r="B12" s="55">
         <v>45487</v>
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="B13" s="56">
+      <c r="B13" s="55">
         <v>45519</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="B14" s="56">
+      <c r="B14" s="55">
         <v>45597</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="B15" s="56">
+      <c r="B15" s="55">
         <v>45607</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="B16" s="56">
+      <c r="B16" s="55">
         <v>45651</v>
       </c>
     </row>
     <row r="17" spans="2:2">
-      <c r="B17" s="56">
+      <c r="B17" s="55">
         <v>45658</v>
       </c>
     </row>
     <row r="18" spans="2:2">
-      <c r="B18" s="56">
+      <c r="B18" s="55">
         <v>45768</v>
       </c>
     </row>
     <row r="19" spans="2:2">
-      <c r="B19" s="56">
+      <c r="B19" s="55">
         <v>45778</v>
       </c>
     </row>
     <row r="20" spans="2:2">
-      <c r="B20" s="56">
+      <c r="B20" s="55">
         <v>45785</v>
       </c>
     </row>
     <row r="21" spans="2:2">
-      <c r="B21" s="56">
+      <c r="B21" s="55">
         <v>45806</v>
       </c>
     </row>
     <row r="22" spans="2:2">
-      <c r="B22" s="56">
+      <c r="B22" s="55">
         <v>45817</v>
       </c>
     </row>
     <row r="23" spans="2:2">
-      <c r="B23" s="56">
+      <c r="B23" s="55">
         <v>45852</v>
       </c>
     </row>
     <row r="24" spans="2:2">
-      <c r="B24" s="56">
+      <c r="B24" s="55">
         <v>45884</v>
       </c>
     </row>
     <row r="25" spans="2:2">
-      <c r="B25" s="56">
+      <c r="B25" s="55">
         <v>45962</v>
       </c>
     </row>
     <row r="26" spans="2:2">
-      <c r="B26" s="56">
+      <c r="B26" s="55">
         <v>45972</v>
       </c>
     </row>
     <row r="27" spans="2:2">
-      <c r="B27" s="56">
+      <c r="B27" s="55">
         <v>46016</v>
       </c>
     </row>
     <row r="28" spans="2:2">
-      <c r="B28" s="56">
+      <c r="B28" s="55">
         <v>46023</v>
       </c>
     </row>
     <row r="29" spans="2:2">
-      <c r="B29" s="56">
+      <c r="B29" s="55">
         <v>46118</v>
       </c>
     </row>
     <row r="30" spans="2:2">
-      <c r="B30" s="56">
+      <c r="B30" s="55">
         <v>46143</v>
       </c>
     </row>
     <row r="31" spans="2:2">
-      <c r="B31" s="56">
+      <c r="B31" s="55">
         <v>46150</v>
       </c>
     </row>
     <row r="32" spans="2:2">
-      <c r="B32" s="56">
+      <c r="B32" s="55">
         <v>46156</v>
       </c>
     </row>
     <row r="33" spans="2:2">
-      <c r="B33" s="56">
+      <c r="B33" s="55">
         <v>46167</v>
       </c>
     </row>
     <row r="34" spans="2:2">
-      <c r="B34" s="56">
+      <c r="B34" s="55">
         <v>46217</v>
       </c>
     </row>
     <row r="35" spans="2:2">
-      <c r="B35" s="56">
+      <c r="B35" s="55">
         <v>46249</v>
       </c>
     </row>
     <row r="36" spans="2:2">
-      <c r="B36" s="56">
+      <c r="B36" s="55">
         <v>46327</v>
       </c>
     </row>
     <row r="37" spans="2:2">
-      <c r="B37" s="56">
+      <c r="B37" s="55">
         <v>46337</v>
       </c>
     </row>
     <row r="38" spans="2:2">
-      <c r="B38" s="56">
+      <c r="B38" s="55">
         <v>46381</v>
       </c>
     </row>
     <row r="39" spans="2:2">
-      <c r="B39" s="56">
+      <c r="B39" s="55">
         <v>46388</v>
       </c>
     </row>
     <row r="40" spans="2:2">
-      <c r="B40" s="56">
+      <c r="B40" s="55">
         <v>46475</v>
       </c>
     </row>
     <row r="41" spans="2:2">
-      <c r="B41" s="56">
+      <c r="B41" s="55">
         <v>46508</v>
       </c>
     </row>
     <row r="42" spans="2:2">
-      <c r="B42" s="56">
+      <c r="B42" s="55">
         <v>46515</v>
       </c>
     </row>
     <row r="43" spans="2:2">
-      <c r="B43" s="56">
+      <c r="B43" s="55">
         <v>46513</v>
       </c>
     </row>
     <row r="44" spans="2:2">
-      <c r="B44" s="56">
+      <c r="B44" s="55">
         <v>46524</v>
       </c>
     </row>
     <row r="45" spans="2:2">
-      <c r="B45" s="56">
+      <c r="B45" s="55">
         <v>46582</v>
       </c>
     </row>
     <row r="46" spans="2:2">
-      <c r="B46" s="56">
+      <c r="B46" s="55">
         <v>46614</v>
       </c>
     </row>
     <row r="47" spans="2:2">
-      <c r="B47" s="56">
+      <c r="B47" s="55">
         <v>46692</v>
       </c>
     </row>
     <row r="48" spans="2:2">
-      <c r="B48" s="56">
+      <c r="B48" s="55">
         <v>46702</v>
       </c>
     </row>
     <row r="49" spans="2:2">
-      <c r="B49" s="56">
+      <c r="B49" s="55">
         <v>46746</v>
       </c>
     </row>
     <row r="50" spans="2:2">
-      <c r="B50" s="56">
+      <c r="B50" s="55">
         <v>46753</v>
       </c>
     </row>
     <row r="51" spans="2:2">
-      <c r="B51" s="56">
+      <c r="B51" s="55">
         <v>46860</v>
       </c>
     </row>
     <row r="52" spans="2:2">
-      <c r="B52" s="56">
+      <c r="B52" s="55">
         <v>46874</v>
       </c>
     </row>
     <row r="53" spans="2:2">
-      <c r="B53" s="56">
+      <c r="B53" s="55">
         <v>46881</v>
       </c>
     </row>
     <row r="54" spans="2:2">
-      <c r="B54" s="56">
+      <c r="B54" s="55">
         <v>46898</v>
       </c>
     </row>
     <row r="55" spans="2:2">
-      <c r="B55" s="56">
+      <c r="B55" s="55">
         <v>46909</v>
       </c>
     </row>
     <row r="56" spans="2:2">
-      <c r="B56" s="56">
+      <c r="B56" s="55">
         <v>46948</v>
       </c>
     </row>
     <row r="57" spans="2:2">
-      <c r="B57" s="56">
+      <c r="B57" s="55">
         <v>46980</v>
       </c>
     </row>
     <row r="58" spans="2:2">
-      <c r="B58" s="56">
+      <c r="B58" s="55">
         <v>47058</v>
       </c>
     </row>
     <row r="59" spans="2:2">
-      <c r="B59" s="56">
+      <c r="B59" s="55">
         <v>47068</v>
       </c>
     </row>
     <row r="60" spans="2:2">
-      <c r="B60" s="56">
+      <c r="B60" s="55">
         <v>47112</v>
       </c>
     </row>
     <row r="61" spans="2:2">
-      <c r="B61" s="56">
+      <c r="B61" s="55">
         <v>47119</v>
       </c>
     </row>
     <row r="62" spans="2:2">
-      <c r="B62" s="56">
+      <c r="B62" s="55">
         <v>47210</v>
       </c>
     </row>
     <row r="63" spans="2:2">
-      <c r="B63" s="56">
+      <c r="B63" s="55">
         <v>47239</v>
       </c>
     </row>
     <row r="64" spans="2:2">
-      <c r="B64" s="56">
+      <c r="B64" s="55">
         <v>47246</v>
       </c>
     </row>
     <row r="65" spans="2:2">
-      <c r="B65" s="56">
+      <c r="B65" s="55">
         <v>47248</v>
       </c>
     </row>
     <row r="66" spans="2:2">
-      <c r="B66" s="56">
+      <c r="B66" s="55">
         <v>47259</v>
       </c>
     </row>
     <row r="67" spans="2:2">
-      <c r="B67" s="56">
+      <c r="B67" s="55">
         <v>47313</v>
       </c>
     </row>
     <row r="68" spans="2:2">
-      <c r="B68" s="56">
+      <c r="B68" s="55">
         <v>47345</v>
       </c>
     </row>
     <row r="69" spans="2:2">
-      <c r="B69" s="56">
+      <c r="B69" s="55">
         <v>47423</v>
       </c>
     </row>
     <row r="70" spans="2:2">
-      <c r="B70" s="56">
+      <c r="B70" s="55">
         <v>47433</v>
       </c>
     </row>
     <row r="71" spans="2:2">
-      <c r="B71" s="56">
+      <c r="B71" s="55">
         <v>47477</v>
       </c>
     </row>
     <row r="72" spans="2:2">
-      <c r="B72" s="56">
+      <c r="B72" s="55">
         <v>47484</v>
       </c>
     </row>
     <row r="73" spans="2:2">
-      <c r="B73" s="56">
+      <c r="B73" s="55">
         <v>47595</v>
       </c>
     </row>
     <row r="74" spans="2:2">
-      <c r="B74" s="56">
+      <c r="B74" s="55">
         <v>47604</v>
       </c>
     </row>
     <row r="75" spans="2:2">
-      <c r="B75" s="56">
+      <c r="B75" s="55">
         <v>47611</v>
       </c>
     </row>
     <row r="76" spans="2:2">
-      <c r="B76" s="56">
+      <c r="B76" s="55">
         <v>47633</v>
       </c>
     </row>
     <row r="77" spans="2:2">
-      <c r="B77" s="56">
+      <c r="B77" s="55">
         <v>47644</v>
       </c>
     </row>
     <row r="78" spans="2:2">
-      <c r="B78" s="56">
+      <c r="B78" s="55">
         <v>47678</v>
       </c>
     </row>
     <row r="79" spans="2:2">
-      <c r="B79" s="56">
+      <c r="B79" s="55">
         <v>47710</v>
       </c>
     </row>
     <row r="80" spans="2:2">
-      <c r="B80" s="56">
+      <c r="B80" s="55">
         <v>47788</v>
       </c>
     </row>
     <row r="81" spans="2:2">
-      <c r="B81" s="56">
+      <c r="B81" s="55">
         <v>47798</v>
       </c>
     </row>
     <row r="82" spans="2:2">
-      <c r="B82" s="56">
+      <c r="B82" s="55">
         <v>47842</v>
       </c>
     </row>
     <row r="83" spans="2:2">
-      <c r="B83" s="56">
+      <c r="B83" s="55">
         <v>47849</v>
       </c>
     </row>
     <row r="84" spans="2:2">
-      <c r="B84" s="56">
+      <c r="B84" s="55">
         <v>47952</v>
       </c>
     </row>
     <row r="85" spans="2:2">
-      <c r="B85" s="56">
+      <c r="B85" s="55">
         <v>47969</v>
       </c>
     </row>
     <row r="86" spans="2:2">
-      <c r="B86" s="56">
+      <c r="B86" s="55">
         <v>47976</v>
       </c>
     </row>
     <row r="87" spans="2:2">
-      <c r="B87" s="56">
+      <c r="B87" s="55">
         <v>47990</v>
       </c>
     </row>
     <row r="88" spans="2:2">
-      <c r="B88" s="56">
+      <c r="B88" s="55">
         <v>48001</v>
       </c>
     </row>
     <row r="89" spans="2:2">
-      <c r="B89" s="56">
+      <c r="B89" s="55">
         <v>48043</v>
       </c>
     </row>
     <row r="90" spans="2:2">
-      <c r="B90" s="56">
+      <c r="B90" s="55">
         <v>48075</v>
       </c>
     </row>
     <row r="91" spans="2:2">
-      <c r="B91" s="56">
+      <c r="B91" s="55">
         <v>48153</v>
       </c>
     </row>
     <row r="92" spans="2:2">
-      <c r="B92" s="56">
+      <c r="B92" s="55">
         <v>48163</v>
       </c>
     </row>
     <row r="93" spans="2:2">
-      <c r="B93" s="56">
+      <c r="B93" s="55">
         <v>48207</v>
       </c>
     </row>
     <row r="94" spans="2:2">
-      <c r="B94" s="56">
+      <c r="B94" s="55">
         <v>48214</v>
       </c>
     </row>
     <row r="95" spans="2:2">
-      <c r="B95" s="56">
+      <c r="B95" s="55">
         <v>48302</v>
       </c>
     </row>
     <row r="96" spans="2:2">
-      <c r="B96" s="56">
+      <c r="B96" s="55">
         <v>48335</v>
       </c>
     </row>
     <row r="97" spans="2:2">
-      <c r="B97" s="56">
+      <c r="B97" s="55">
         <v>48342</v>
       </c>
     </row>
     <row r="98" spans="2:2">
-      <c r="B98" s="56">
+      <c r="B98" s="55">
         <v>48340</v>
       </c>
     </row>
     <row r="99" spans="2:2">
-      <c r="B99" s="56">
+      <c r="B99" s="55">
         <v>48351</v>
       </c>
     </row>
     <row r="100" spans="2:2">
-      <c r="B100" s="56">
+      <c r="B100" s="55">
         <v>48409</v>
       </c>
     </row>
     <row r="101" spans="2:2">
-      <c r="B101" s="56">
+      <c r="B101" s="55">
         <v>48441</v>
       </c>
     </row>
     <row r="102" spans="2:2">
-      <c r="B102" s="56">
+      <c r="B102" s="55">
         <v>48519</v>
       </c>
     </row>
     <row r="103" spans="2:2">
-      <c r="B103" s="56">
+      <c r="B103" s="55">
         <v>48529</v>
       </c>
     </row>
     <row r="104" spans="2:2">
-      <c r="B104" s="56">
+      <c r="B104" s="55">
         <v>48573</v>
       </c>
     </row>
     <row r="105" spans="2:2">
-      <c r="B105" s="56">
+      <c r="B105" s="55">
         <v>48580</v>
       </c>
     </row>
     <row r="106" spans="2:2">
-      <c r="B106" s="56">
+      <c r="B106" s="55">
         <v>48687</v>
       </c>
     </row>
     <row r="107" spans="2:2">
-      <c r="B107" s="56">
+      <c r="B107" s="55">
         <v>48700</v>
       </c>
     </row>
     <row r="108" spans="2:2">
-      <c r="B108" s="56">
+      <c r="B108" s="55">
         <v>48707</v>
       </c>
     </row>
     <row r="109" spans="2:2">
-      <c r="B109" s="56">
+      <c r="B109" s="55">
         <v>48725</v>
       </c>
     </row>
     <row r="110" spans="2:2">
-      <c r="B110" s="56">
+      <c r="B110" s="55">
         <v>48736</v>
       </c>
     </row>
     <row r="111" spans="2:2">
-      <c r="B111" s="56">
+      <c r="B111" s="55">
         <v>48774</v>
       </c>
     </row>
     <row r="112" spans="2:2">
-      <c r="B112" s="56">
+      <c r="B112" s="55">
         <v>48806</v>
       </c>
     </row>
     <row r="113" spans="2:2">
-      <c r="B113" s="56">
+      <c r="B113" s="55">
         <v>48884</v>
       </c>
     </row>
     <row r="114" spans="2:2">
-      <c r="B114" s="56">
+      <c r="B114" s="55">
         <v>48894</v>
       </c>
     </row>
     <row r="115" spans="2:2">
-      <c r="B115" s="56">
+      <c r="B115" s="55">
         <v>48938</v>
       </c>
     </row>
     <row r="116" spans="2:2">
-      <c r="B116" s="56">
+      <c r="B116" s="55">
         <v>48945</v>
       </c>
     </row>
     <row r="117" spans="2:2">
-      <c r="B117" s="56">
+      <c r="B117" s="55">
         <v>49044</v>
       </c>
     </row>
     <row r="118" spans="2:2">
-      <c r="B118" s="56">
+      <c r="B118" s="55">
         <v>49065</v>
       </c>
     </row>
     <row r="119" spans="2:2">
-      <c r="B119" s="56">
+      <c r="B119" s="55">
         <v>49072</v>
       </c>
     </row>
     <row r="120" spans="2:2">
-      <c r="B120" s="56">
+      <c r="B120" s="55">
         <v>49082</v>
       </c>
     </row>
     <row r="121" spans="2:2">
-      <c r="B121" s="56">
+      <c r="B121" s="55">
         <v>49093</v>
       </c>
     </row>
     <row r="122" spans="2:2">
-      <c r="B122" s="56">
+      <c r="B122" s="55">
         <v>49139</v>
       </c>
     </row>
     <row r="123" spans="2:2">
-      <c r="B123" s="56">
+      <c r="B123" s="55">
         <v>49171</v>
       </c>
     </row>
     <row r="124" spans="2:2">
-      <c r="B124" s="56">
+      <c r="B124" s="55">
         <v>49249</v>
       </c>
     </row>
     <row r="125" spans="2:2">
-      <c r="B125" s="56">
+      <c r="B125" s="55">
         <v>49259</v>
       </c>
     </row>
     <row r="126" spans="2:2">
-      <c r="B126" s="56">
+      <c r="B126" s="55">
         <v>49303</v>
       </c>
     </row>
     <row r="127" spans="2:2">
-      <c r="B127" s="56">
+      <c r="B127" s="55">
         <v>49310</v>
       </c>
     </row>
     <row r="128" spans="2:2">
-      <c r="B128" s="56">
+      <c r="B128" s="55">
         <v>49394</v>
       </c>
     </row>
     <row r="129" spans="2:2">
-      <c r="B129" s="56">
+      <c r="B129" s="55">
         <v>49430</v>
       </c>
     </row>
     <row r="130" spans="2:2">
-      <c r="B130" s="56">
+      <c r="B130" s="55">
         <v>49437</v>
       </c>
     </row>
     <row r="131" spans="2:2">
-      <c r="B131" s="56">
+      <c r="B131" s="55">
         <v>49432</v>
       </c>
     </row>
     <row r="132" spans="2:2">
-      <c r="B132" s="56">
+      <c r="B132" s="55">
         <v>49443</v>
       </c>
     </row>
     <row r="133" spans="2:2">
-      <c r="B133" s="56">
+      <c r="B133" s="55">
         <v>49504</v>
       </c>
     </row>
     <row r="134" spans="2:2">
-      <c r="B134" s="56">
+      <c r="B134" s="55">
         <v>49536</v>
       </c>
     </row>
     <row r="135" spans="2:2">
-      <c r="B135" s="56">
+      <c r="B135" s="55">
         <v>49614</v>
       </c>
     </row>
     <row r="136" spans="2:2">
-      <c r="B136" s="56">
+      <c r="B136" s="55">
         <v>49624</v>
       </c>
     </row>
     <row r="137" spans="2:2">
-      <c r="B137" s="56">
+      <c r="B137" s="55">
         <v>49668</v>
       </c>
     </row>
     <row r="138" spans="2:2">
-      <c r="B138" s="56">
+      <c r="B138" s="55">
         <v>49675</v>
       </c>
     </row>
     <row r="139" spans="2:2">
-      <c r="B139" s="56">
+      <c r="B139" s="55">
         <v>49779</v>
       </c>
     </row>
     <row r="140" spans="2:2">
-      <c r="B140" s="56">
+      <c r="B140" s="55">
         <v>49796</v>
       </c>
     </row>
     <row r="141" spans="2:2">
-      <c r="B141" s="56">
+      <c r="B141" s="55">
         <v>49803</v>
       </c>
     </row>
     <row r="142" spans="2:2">
-      <c r="B142" s="56">
+      <c r="B142" s="55">
         <v>49817</v>
       </c>
     </row>
     <row r="143" spans="2:2">
-      <c r="B143" s="56">
+      <c r="B143" s="55">
         <v>49828</v>
       </c>
     </row>
     <row r="144" spans="2:2">
-      <c r="B144" s="56">
+      <c r="B144" s="55">
         <v>49870</v>
       </c>
     </row>
     <row r="145" spans="2:2">
-      <c r="B145" s="56">
+      <c r="B145" s="55">
         <v>49902</v>
       </c>
     </row>
     <row r="146" spans="2:2">
-      <c r="B146" s="56">
+      <c r="B146" s="55">
         <v>49980</v>
       </c>
     </row>
     <row r="147" spans="2:2">
-      <c r="B147" s="56">
+      <c r="B147" s="55">
         <v>49990</v>
       </c>
     </row>
     <row r="148" spans="2:2">
-      <c r="B148" s="56">
+      <c r="B148" s="55">
         <v>50034</v>
       </c>
     </row>
     <row r="149" spans="2:2">
-      <c r="B149" s="56">
+      <c r="B149" s="55">
         <v>50041</v>
       </c>
     </row>
     <row r="150" spans="2:2">
-      <c r="B150" s="56">
+      <c r="B150" s="55">
         <v>50136</v>
       </c>
     </row>
     <row r="151" spans="2:2">
-      <c r="B151" s="56">
+      <c r="B151" s="55">
         <v>50161</v>
       </c>
     </row>
     <row r="152" spans="2:2">
-      <c r="B152" s="56">
+      <c r="B152" s="55">
         <v>50168</v>
       </c>
     </row>
     <row r="153" spans="2:2">
-      <c r="B153" s="56">
+      <c r="B153" s="55">
         <v>50174</v>
       </c>
     </row>
     <row r="154" spans="2:2">
-      <c r="B154" s="56">
+      <c r="B154" s="55">
         <v>50185</v>
       </c>
     </row>
     <row r="155" spans="2:2">
-      <c r="B155" s="56">
+      <c r="B155" s="55">
         <v>50235</v>
       </c>
     </row>
     <row r="156" spans="2:2">
-      <c r="B156" s="56">
+      <c r="B156" s="55">
         <v>50267</v>
       </c>
     </row>
     <row r="157" spans="2:2">
-      <c r="B157" s="56">
+      <c r="B157" s="55">
         <v>50345</v>
       </c>
     </row>
     <row r="158" spans="2:2">
-      <c r="B158" s="56">
+      <c r="B158" s="55">
         <v>50355</v>
       </c>
     </row>
     <row r="159" spans="2:2">
-      <c r="B159" s="56">
+      <c r="B159" s="55">
         <v>50399</v>
       </c>
     </row>
     <row r="160" spans="2:2">
-      <c r="B160" s="56">
+      <c r="B160" s="55">
         <v>50406</v>
       </c>
     </row>
     <row r="161" spans="2:2">
-      <c r="B161" s="56">
+      <c r="B161" s="55">
         <v>50521</v>
       </c>
     </row>
     <row r="162" spans="2:2">
-      <c r="B162" s="56">
+      <c r="B162" s="55">
         <v>50526</v>
       </c>
     </row>
     <row r="163" spans="2:2">
-      <c r="B163" s="56">
+      <c r="B163" s="55">
         <v>50533</v>
       </c>
     </row>
     <row r="164" spans="2:2">
-      <c r="B164" s="56">
+      <c r="B164" s="55">
         <v>50559</v>
       </c>
     </row>
     <row r="165" spans="2:2">
-      <c r="B165" s="56">
+      <c r="B165" s="55">
         <v>50570</v>
       </c>
     </row>
     <row r="166" spans="2:2">
-      <c r="B166" s="56">
+      <c r="B166" s="55">
         <v>50600</v>
       </c>
     </row>
     <row r="167" spans="2:2">
-      <c r="B167" s="56">
+      <c r="B167" s="55">
         <v>50632</v>
       </c>
     </row>
     <row r="168" spans="2:2">
-      <c r="B168" s="56">
+      <c r="B168" s="55">
         <v>50710</v>
       </c>
     </row>
     <row r="169" spans="2:2">
-      <c r="B169" s="56">
+      <c r="B169" s="55">
         <v>50720</v>
       </c>
     </row>
     <row r="170" spans="2:2">
-      <c r="B170" s="56">
+      <c r="B170" s="55">
         <v>50764</v>
       </c>
     </row>
     <row r="171" spans="2:2">
-      <c r="B171" s="56">
+      <c r="B171" s="55">
         <v>50771</v>
       </c>
     </row>
     <row r="172" spans="2:2">
-      <c r="B172" s="56">
+      <c r="B172" s="55">
         <v>50871</v>
       </c>
     </row>
     <row r="173" spans="2:2">
-      <c r="B173" s="56">
+      <c r="B173" s="55">
         <v>50891</v>
       </c>
     </row>
     <row r="174" spans="2:2">
-      <c r="B174" s="56">
+      <c r="B174" s="55">
         <v>50898</v>
       </c>
     </row>
     <row r="175" spans="2:2">
-      <c r="B175" s="56">
+      <c r="B175" s="55">
         <v>50909</v>
       </c>
     </row>
     <row r="176" spans="2:2">
-      <c r="B176" s="56">
+      <c r="B176" s="55">
         <v>50920</v>
       </c>
     </row>
     <row r="177" spans="2:2">
-      <c r="B177" s="56">
+      <c r="B177" s="55">
         <v>50965</v>
       </c>
     </row>
     <row r="178" spans="2:2">
-      <c r="B178" s="56">
+      <c r="B178" s="55">
         <v>50997</v>
       </c>
     </row>
     <row r="179" spans="2:2">
-      <c r="B179" s="56">
+      <c r="B179" s="55">
         <v>51075</v>
       </c>
     </row>
     <row r="180" spans="2:2">
-      <c r="B180" s="56">
+      <c r="B180" s="55">
         <v>51085</v>
       </c>
     </row>
     <row r="181" spans="2:2">
-      <c r="B181" s="56">
+      <c r="B181" s="55">
         <v>51129</v>
       </c>
     </row>
     <row r="182" spans="2:2">
-      <c r="B182" s="56">
+      <c r="B182" s="55">
         <v>51136</v>
       </c>
     </row>
     <row r="183" spans="2:2">
-      <c r="B183" s="56">
+      <c r="B183" s="55">
         <v>51228</v>
       </c>
     </row>
     <row r="184" spans="2:2">
-      <c r="B184" s="56">
+      <c r="B184" s="55">
         <v>51257</v>
       </c>
     </row>
     <row r="185" spans="2:2">
-      <c r="B185" s="56">
+      <c r="B185" s="55">
         <v>51264</v>
       </c>
     </row>
     <row r="186" spans="2:2">
-      <c r="B186" s="56">
+      <c r="B186" s="55">
         <v>51266</v>
       </c>
     </row>
     <row r="187" spans="2:2">
-      <c r="B187" s="56">
+      <c r="B187" s="55">
         <v>51277</v>
       </c>
     </row>
     <row r="188" spans="2:2">
-      <c r="B188" s="56">
+      <c r="B188" s="55">
         <v>51331</v>
       </c>
     </row>
     <row r="189" spans="2:2">
-      <c r="B189" s="56">
+      <c r="B189" s="55">
         <v>51363</v>
       </c>
     </row>
     <row r="190" spans="2:2">
-      <c r="B190" s="56">
+      <c r="B190" s="55">
         <v>51441</v>
       </c>
     </row>
     <row r="191" spans="2:2">
-      <c r="B191" s="56">
+      <c r="B191" s="55">
         <v>51451</v>
       </c>
     </row>
     <row r="192" spans="2:2">
-      <c r="B192" s="56">
+      <c r="B192" s="55">
         <v>51495</v>
       </c>
     </row>
     <row r="193" spans="2:2">
-      <c r="B193" s="56">
+      <c r="B193" s="55">
         <v>51502</v>
       </c>
     </row>
     <row r="194" spans="2:2">
-      <c r="B194" s="56">
+      <c r="B194" s="55">
         <v>51613</v>
       </c>
     </row>
     <row r="195" spans="2:2">
-      <c r="B195" s="56">
+      <c r="B195" s="55">
         <v>51622</v>
       </c>
     </row>
     <row r="196" spans="2:2">
-      <c r="B196" s="56">
+      <c r="B196" s="55">
         <v>51629</v>
       </c>
     </row>
     <row r="197" spans="2:2">
-      <c r="B197" s="56">
+      <c r="B197" s="55">
         <v>51651</v>
       </c>
     </row>
     <row r="198" spans="2:2">
-      <c r="B198" s="56">
+      <c r="B198" s="55">
         <v>51662</v>
       </c>
     </row>
     <row r="199" spans="2:2">
-      <c r="B199" s="56">
+      <c r="B199" s="55">
         <v>51696</v>
       </c>
     </row>
     <row r="200" spans="2:2">
-      <c r="B200" s="56">
+      <c r="B200" s="55">
         <v>51728</v>
       </c>
     </row>
     <row r="201" spans="2:2">
-      <c r="B201" s="56">
+      <c r="B201" s="55">
         <v>51806</v>
       </c>
     </row>
     <row r="202" spans="2:2">
-      <c r="B202" s="56">
+      <c r="B202" s="55">
         <v>51816</v>
       </c>
     </row>
     <row r="203" spans="2:2">
-      <c r="B203" s="56">
+      <c r="B203" s="55">
         <v>51860</v>
       </c>
     </row>
     <row r="204" spans="2:2">
-      <c r="B204" s="56">
+      <c r="B204" s="55">
         <v>51867</v>
       </c>
     </row>
     <row r="205" spans="2:2">
-      <c r="B205" s="56">
+      <c r="B205" s="55">
         <v>51963</v>
       </c>
     </row>
     <row r="206" spans="2:2">
-      <c r="B206" s="56">
+      <c r="B206" s="55">
         <v>51987</v>
       </c>
     </row>
     <row r="207" spans="2:2">
-      <c r="B207" s="56">
+      <c r="B207" s="55">
         <v>51994</v>
       </c>
     </row>
     <row r="208" spans="2:2">
-      <c r="B208" s="56">
+      <c r="B208" s="55">
         <v>52001</v>
       </c>
     </row>
     <row r="209" spans="2:2">
-      <c r="B209" s="56">
+      <c r="B209" s="55">
         <v>52012</v>
       </c>
     </row>
     <row r="210" spans="2:2">
-      <c r="B210" s="56">
+      <c r="B210" s="55">
         <v>52061</v>
       </c>
     </row>
     <row r="211" spans="2:2">
-      <c r="B211" s="56">
+      <c r="B211" s="55">
         <v>52093</v>
       </c>
     </row>
     <row r="212" spans="2:2">
-      <c r="B212" s="56">
+      <c r="B212" s="55">
         <v>52171</v>
       </c>
     </row>
     <row r="213" spans="2:2">
-      <c r="B213" s="56">
+      <c r="B213" s="55">
         <v>52181</v>
       </c>
     </row>
     <row r="214" spans="2:2">
-      <c r="B214" s="56">
+      <c r="B214" s="55">
         <v>52225</v>
       </c>
     </row>
     <row r="215" spans="2:2">
-      <c r="B215" s="56">
+      <c r="B215" s="55">
         <v>52232</v>
       </c>
     </row>
     <row r="216" spans="2:2">
-      <c r="B216" s="56">
+      <c r="B216" s="55">
         <v>52320</v>
       </c>
     </row>
     <row r="217" spans="2:2">
-      <c r="B217" s="56">
+      <c r="B217" s="55">
         <v>52352</v>
       </c>
     </row>
     <row r="218" spans="2:2">
-      <c r="B218" s="56">
+      <c r="B218" s="55">
         <v>52359</v>
       </c>
     </row>
     <row r="219" spans="2:2">
-      <c r="B219" s="56">
+      <c r="B219" s="55">
         <v>52358</v>
       </c>
     </row>
     <row r="220" spans="2:2">
-      <c r="B220" s="56">
+      <c r="B220" s="55">
         <v>52369</v>
       </c>
     </row>
     <row r="221" spans="2:2">
-      <c r="B221" s="56">
+      <c r="B221" s="55">
         <v>52426</v>
       </c>
     </row>
     <row r="222" spans="2:2">
-      <c r="B222" s="56">
+      <c r="B222" s="55">
         <v>52458</v>
       </c>
     </row>
     <row r="223" spans="2:2">
-      <c r="B223" s="56">
+      <c r="B223" s="55">
         <v>52536</v>
       </c>
     </row>
     <row r="224" spans="2:2">
-      <c r="B224" s="56">
+      <c r="B224" s="55">
         <v>52546</v>
       </c>
     </row>
     <row r="225" spans="2:2">
-      <c r="B225" s="56">
+      <c r="B225" s="55">
         <v>52590</v>
       </c>
     </row>
     <row r="226" spans="2:2">
-      <c r="B226" s="56">
+      <c r="B226" s="55">
         <v>52597</v>
       </c>
     </row>
     <row r="227" spans="2:2">
-      <c r="B227" s="56">
+      <c r="B227" s="55">
         <v>52705</v>
       </c>
     </row>
     <row r="228" spans="2:2">
-      <c r="B228" s="56">
+      <c r="B228" s="55">
         <v>52718</v>
       </c>
     </row>
     <row r="229" spans="2:2">
-      <c r="B229" s="56">
+      <c r="B229" s="55">
         <v>52725</v>
       </c>
     </row>
     <row r="230" spans="2:2">
-      <c r="B230" s="56">
+      <c r="B230" s="55">
         <v>52743</v>
       </c>
     </row>
     <row r="231" spans="2:2">
-      <c r="B231" s="56">
+      <c r="B231" s="55">
         <v>52754</v>
       </c>
     </row>
     <row r="232" spans="2:2">
-      <c r="B232" s="56">
+      <c r="B232" s="55">
         <v>52792</v>
       </c>
     </row>
     <row r="233" spans="2:2">
-      <c r="B233" s="56">
+      <c r="B233" s="55">
         <v>52824</v>
       </c>
     </row>
     <row r="234" spans="2:2">
-      <c r="B234" s="56">
+      <c r="B234" s="55">
         <v>52902</v>
       </c>
     </row>
     <row r="235" spans="2:2">
-      <c r="B235" s="56">
+      <c r="B235" s="55">
         <v>52912</v>
       </c>
     </row>
     <row r="236" spans="2:2">
-      <c r="B236" s="56">
+      <c r="B236" s="55">
         <v>52956</v>
       </c>
     </row>
     <row r="237" spans="2:2">
-      <c r="B237" s="56">
+      <c r="B237" s="55">
         <v>52963</v>
       </c>
     </row>
     <row r="238" spans="2:2">
-      <c r="B238" s="56">
+      <c r="B238" s="55">
         <v>53062</v>
       </c>
     </row>
     <row r="239" spans="2:2">
-      <c r="B239" s="56">
+      <c r="B239" s="55">
         <v>53083</v>
       </c>
     </row>
     <row r="240" spans="2:2">
-      <c r="B240" s="56">
+      <c r="B240" s="55">
         <v>53090</v>
       </c>
     </row>
     <row r="241" spans="2:2">
-      <c r="B241" s="56">
+      <c r="B241" s="55">
         <v>53100</v>
       </c>
     </row>
     <row r="242" spans="2:2">
-      <c r="B242" s="56">
+      <c r="B242" s="55">
         <v>53111</v>
       </c>
     </row>
     <row r="243" spans="2:2">
-      <c r="B243" s="56">
+      <c r="B243" s="55">
         <v>53157</v>
       </c>
     </row>
     <row r="244" spans="2:2">
-      <c r="B244" s="56">
+      <c r="B244" s="55">
         <v>53189</v>
       </c>
     </row>
     <row r="245" spans="2:2">
-      <c r="B245" s="56">
+      <c r="B245" s="55">
         <v>53267</v>
       </c>
     </row>
     <row r="246" spans="2:2">
-      <c r="B246" s="56">
+      <c r="B246" s="55">
         <v>53277</v>
       </c>
     </row>
     <row r="247" spans="2:2">
-      <c r="B247" s="56">
+      <c r="B247" s="55">
         <v>53321</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refait l'interface du classeur à macros en formes, comme le site
Cartes arrondies avec ombre, cases, diodes, frise, pastilles et icônes de copie
sont des formes décrites dans la feuille Rendu (excel/interface.py) ; un moteur VBA
générique les crée et ne met à jour que ce qui change. Les champs de saisie restent
de vraies cellules sous des formes qui s'effacent pendant la frappe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Racco_D2.xlsx
+++ b/excel/Racco_D2.xlsx
@@ -41,6 +41,9 @@
     <definedName name="sel">'Calcul'!$B$52:$B$52</definedName>
     <definedName name="selMemo">'Calcul'!$B$54:$B$54</definedName>
     <definedName name="taches">'Calcul'!$A$43:$R$49</definedName>
+    <definedName name="v_cab">'Racco D2'!$V$7:$V$7</definedName>
+    <definedName name="v_dep">'Racco D2'!$H$29:$H$29</definedName>
+    <definedName name="v_dlpi">'Racco D2'!$AC$7:$AC$7</definedName>
     <definedName name="vue">'Calcul'!$B$53:$B$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="170">
   <si>
     <t>Paramètres</t>
   </si>
@@ -411,6 +414,9 @@
   </si>
   <si>
     <t>étape mémorisée</t>
+  </si>
+  <si>
+    <t>étape choisie</t>
   </si>
   <si>
     <t>Code Comlab</t>
@@ -1525,7 +1531,7 @@
     <row r="2" spans="2:37" ht="6" customHeight="1"/>
     <row r="3" spans="2:37" ht="18" customHeight="1">
       <c r="B3" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -1535,7 +1541,7 @@
       </c>
       <c r="F3" s="6"/>
       <c r="H3" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
@@ -1577,10 +1583,10 @@
         <v>22</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
@@ -1589,7 +1595,7 @@
       <c r="M4" s="13"/>
       <c r="N4" s="13"/>
       <c r="O4" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
@@ -1598,7 +1604,7 @@
       <c r="T4" s="13"/>
       <c r="U4" s="13"/>
       <c r="V4" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="W4" s="13"/>
       <c r="X4" s="13"/>
@@ -1607,7 +1613,7 @@
       <c r="AA4" s="13"/>
       <c r="AB4" s="13"/>
       <c r="AC4" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AD4" s="13"/>
       <c r="AE4" s="13"/>
@@ -1672,7 +1678,7 @@
       </c>
       <c r="F6" s="19"/>
       <c r="H6" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13"/>
@@ -1688,7 +1694,7 @@
       <c r="T6" s="13"/>
       <c r="U6" s="13"/>
       <c r="V6" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="W6" s="13"/>
       <c r="X6" s="13"/>
@@ -1697,7 +1703,7 @@
       <c r="AA6" s="13"/>
       <c r="AB6" s="13"/>
       <c r="AC6" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="AD6" s="13"/>
       <c r="AE6" s="13"/>
@@ -1762,7 +1768,7 @@
       </c>
       <c r="F8" s="19"/>
       <c r="H8" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I8" s="13"/>
       <c r="J8" s="13"/>
@@ -1807,7 +1813,7 @@
         <v>33</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H9" s="23"/>
       <c r="I9" s="23"/>
@@ -1908,7 +1914,7 @@
       </c>
       <c r="F12" s="19"/>
       <c r="H12" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
@@ -1929,7 +1935,7 @@
       <c r="V12" s="25"/>
       <c r="W12" s="6"/>
       <c r="X12" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Y12" s="26"/>
       <c r="Z12" s="26"/>
@@ -2007,7 +2013,7 @@
       <c r="C14" s="29"/>
       <c r="D14" s="29"/>
       <c r="E14" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F14" s="29"/>
       <c r="H14" s="31" t="s">
@@ -2053,7 +2059,7 @@
       <c r="AH14" s="31"/>
       <c r="AI14" s="31"/>
       <c r="AK14" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="2:37" ht="18" customHeight="1">
@@ -2115,7 +2121,7 @@
       </c>
       <c r="F16" s="19"/>
       <c r="H16" s="34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I16" s="34"/>
       <c r="J16" s="34"/>
@@ -2162,7 +2168,7 @@
       </c>
       <c r="F17" s="19"/>
       <c r="H17" s="34" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="34"/>
@@ -2210,10 +2216,10 @@
         <v>52</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="34"/>
@@ -2386,7 +2392,7 @@
       </c>
       <c r="F22" s="19"/>
       <c r="H22" s="34" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I22" s="34"/>
       <c r="J22" s="34"/>
@@ -2434,10 +2440,10 @@
         <v>62</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I23" s="34"/>
       <c r="J23" s="34"/>
@@ -2445,7 +2451,7 @@
       <c r="L23" s="34"/>
       <c r="M23" s="34"/>
       <c r="N23" s="35">
-        <f>IF('Racco D2'!$AC$7="","DLPI non renseignée",IF('Racco D2'!$AC$7-TODAY()&gt;0,"J-"&amp;('Racco D2'!$AC$7-TODAY())&amp;" avant la DLPI",IF('Racco D2'!$AC$7-TODAY()=0,"DLPI aujourd'hui","DLPI dépassée de "&amp;(TODAY()-'Racco D2'!$AC$7)&amp;" j")))</f>
+        <f>IF(v_dlpi="","DLPI non renseignée",IF(v_dlpi-TODAY()&gt;0,"J-"&amp;(v_dlpi-TODAY())&amp;" avant la DLPI",IF(v_dlpi-TODAY()=0,"DLPI aujourd'hui","DLPI dépassée de "&amp;(TODAY()-v_dlpi)&amp;" j")))</f>
         <v>0</v>
       </c>
       <c r="O23" s="35"/>
@@ -2586,10 +2592,10 @@
         <v>70</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
@@ -2633,7 +2639,7 @@
       </c>
       <c r="F28" s="19"/>
       <c r="H28" s="37" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I28" s="37"/>
       <c r="J28" s="37"/>
@@ -2645,7 +2651,7 @@
       <c r="P28" s="37"/>
       <c r="Q28" s="37"/>
       <c r="R28" s="37" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="S28" s="37"/>
       <c r="T28" s="37"/>
@@ -2656,7 +2662,7 @@
       <c r="Y28" s="29"/>
       <c r="Z28" s="29"/>
       <c r="AA28" s="37" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB28" s="37"/>
       <c r="AC28" s="37"/>
@@ -2823,7 +2829,7 @@
         <v>80</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
@@ -2868,7 +2874,7 @@
       </c>
       <c r="F33" s="19"/>
       <c r="H33" s="42" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I33" s="42"/>
       <c r="J33" s="42"/>
@@ -2912,7 +2918,7 @@
       </c>
       <c r="F34" s="19"/>
       <c r="H34" s="37" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I34" s="37"/>
       <c r="J34" s="37"/>
@@ -2928,7 +2934,7 @@
       <c r="T34" s="29"/>
       <c r="U34" s="29"/>
       <c r="V34" s="37" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="W34" s="37"/>
       <c r="X34" s="37"/>
@@ -3006,7 +3012,7 @@
       <c r="C36" s="29"/>
       <c r="D36" s="29"/>
       <c r="E36" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F36" s="29"/>
       <c r="H36" s="43"/>
@@ -3038,7 +3044,7 @@
       <c r="AH36" s="43"/>
       <c r="AI36" s="43"/>
       <c r="AK36" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37" spans="2:37" ht="18" customHeight="1">
@@ -3052,7 +3058,7 @@
       </c>
       <c r="F37" s="19"/>
       <c r="H37" s="45" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I37" s="45"/>
       <c r="J37" s="45"/>
@@ -3184,10 +3190,10 @@
         <v>96</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H40" s="47" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I40" s="47"/>
       <c r="J40" s="47"/>
@@ -3206,7 +3212,7 @@
       <c r="T40" s="29"/>
       <c r="U40" s="29"/>
       <c r="V40" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="W40" s="47"/>
       <c r="X40" s="47"/>
@@ -3281,7 +3287,7 @@
       </c>
       <c r="F42" s="19"/>
       <c r="H42" s="47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I42" s="47"/>
       <c r="J42" s="47"/>
@@ -3300,7 +3306,7 @@
       <c r="T42" s="29"/>
       <c r="U42" s="29"/>
       <c r="V42" s="47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="W42" s="47"/>
       <c r="X42" s="47"/>
@@ -5607,7 +5613,7 @@
         <v>0</v>
       </c>
       <c r="Q43">
-        <f>IF(I43,"—",IF(D43,"Moi",IF(TRUE,IF('Racco D2'!$V$7="","Cabinet conseil",'Racco D2'!$V$7),IF('Racco D2'!$V$7="","Cabinet conseil",'Racco D2'!$V$7))))</f>
+        <f>IF(I43,"—",IF(D43,"Moi",IF(TRUE,IF(v_cab="","Cabinet conseil",v_cab),IF(v_cab="","Cabinet conseil",v_cab))))</f>
         <v>0</v>
       </c>
       <c r="R43">
@@ -5678,7 +5684,7 @@
         <v>0</v>
       </c>
       <c r="Q44">
-        <f>IF(I44,"—",IF(E44,"Moi",IF(F44,IF('Racco D2'!$V$7="","Cabinet conseil",'Racco D2'!$V$7),IF(AND(Calcul!$E$7,NOT(G44),NOT(H44)),"Moi",IF(G44,"Moi",IF(H44,"Moi","Moi"))))))</f>
+        <f>IF(I44,"—",IF(E44,"Moi",IF(F44,IF(v_cab="","Cabinet conseil",v_cab),IF(AND(Calcul!$E$7,NOT(G44),NOT(H44)),"Moi",IF(G44,"Moi",IF(H44,"Moi","Moi"))))))</f>
         <v>0</v>
       </c>
       <c r="R44">
@@ -6008,14 +6014,19 @@
         <v>120</v>
       </c>
     </row>
+    <row r="55" spans="1:18">
+      <c r="A55" t="s">
+        <v>121</v>
+      </c>
+    </row>
     <row r="57" spans="1:18">
       <c r="A57" s="49" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="58" spans="1:18">
       <c r="A58" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B58">
         <f>Calcul!$R$43&amp;Calcul!$R$44&amp;Calcul!$R$45&amp;Calcul!$R$46&amp;Calcul!$R$47&amp;Calcul!$R$48&amp;Calcul!$R$49&amp;MID('Paramètres'!$D$2,1+16*N(Calcul!$F$3)+8*N(Calcul!$F$4)+4*N(Calcul!$F$5)+2*N(Calcul!$F$6)+1*N(Calcul!$F$9),1)&amp;MID('Paramètres'!$D$2,1+16*N(Calcul!$F$10)+8*N(Calcul!$F$11)+4*N(Calcul!$F$13)+2*N(Calcul!$F$14)+1*N(Calcul!$F$16),1)&amp;MID('Paramètres'!$D$2,1+16*N(Calcul!$F$17)+8*N(Calcul!$F$18)+4*N(Calcul!$F$19)+2*N(Calcul!$F$21)+1*N(Calcul!$F$22),1)&amp;MID('Paramètres'!$D$2,1+16*N(Calcul!$F$23)+8*N(Calcul!$F$25)+4*N(Calcul!$F$26)+2*N(Calcul!$F$27)+1*N(Calcul!$F$28),1)&amp;MID('Paramètres'!$D$2,1+16*N(Calcul!$F$31)+8*N(Calcul!$F$32)+4*N(Calcul!$F$34)+2*N(Calcul!$F$35)+1*N(Calcul!$F$37),1)&amp;MID('Paramètres'!$D$2,1+16*N(Calcul!$F$38)+8*N(Calcul!$F$39),1)&amp;MID('Paramètres'!$D$2,1+0,1)&amp;MID('Paramètres'!$D$2,1+0,1)&amp;MID('Paramètres'!$D$2,1+0,1)&amp;MID('Paramètres'!$D$2,1+0,1)&amp;MID('Paramètres'!$D$2,1+0,1)&amp;MID('Paramètres'!$D$2,1+0,1)&amp;MID('Paramètres'!$D$2,1+0,1)&amp;MID('Paramètres'!$D$2,1+0,1)</f>
@@ -6024,13 +6035,13 @@
     </row>
     <row r="59" spans="1:18">
       <c r="A59" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B59" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C59" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="60" spans="1:18">
@@ -6308,7 +6319,7 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B82">
         <f>Calcul!$B$58&amp;MID('Paramètres'!$D$2,MOD(INT(C80/1),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C80/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C80/1024),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C80/32768),32)+1,1)</f>
@@ -6317,12 +6328,12 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="49" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B86">
         <f>"ape"&amp;Calcul!$B$82&amp;0</f>
@@ -6621,7 +6632,7 @@
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B116">
         <f>"ape"&amp;Calcul!$B$82&amp;2</f>
@@ -6920,7 +6931,7 @@
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B146">
         <f>"ape"&amp;Calcul!$B$82&amp;4</f>
@@ -7219,7 +7230,7 @@
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B176">
         <f>"ape"&amp;Calcul!$B$82&amp;6</f>
@@ -7518,7 +7529,7 @@
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B206">
         <f>"ape"&amp;Calcul!$B$82&amp;8</f>
@@ -7817,7 +7828,7 @@
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B236">
         <f>"ape"&amp;Calcul!$B$82&amp;10</f>
@@ -8126,7 +8137,7 @@
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B267">
         <f>"ape"&amp;Calcul!$B$82&amp;12</f>
@@ -8435,7 +8446,7 @@
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B298">
         <f>"ape"&amp;Calcul!$B$82&amp;14</f>
@@ -8744,7 +8755,7 @@
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B329">
         <f>LEFT(MID('Paramètres'!$D$2,MOD(C115,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C115/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C145,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C145/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C175,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C175/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C205,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C205/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C235,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C235/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C266,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C266/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C297,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C297/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C328,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C328/32),32)+1,1),15)</f>
@@ -8753,12 +8764,12 @@
     </row>
     <row r="331" spans="1:3">
       <c r="A331" s="49" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B332">
         <f>"dzi"&amp;Calcul!$B$82&amp;0</f>
@@ -9057,7 +9068,7 @@
     </row>
     <row r="362" spans="1:3">
       <c r="A362" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B362">
         <f>"dzi"&amp;Calcul!$B$82&amp;2</f>
@@ -9356,7 +9367,7 @@
     </row>
     <row r="392" spans="1:3">
       <c r="A392" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B392">
         <f>"dzi"&amp;Calcul!$B$82&amp;4</f>
@@ -9655,7 +9666,7 @@
     </row>
     <row r="422" spans="1:3">
       <c r="A422" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B422">
         <f>"dzi"&amp;Calcul!$B$82&amp;6</f>
@@ -9954,7 +9965,7 @@
     </row>
     <row r="452" spans="1:3">
       <c r="A452" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B452">
         <f>"dzi"&amp;Calcul!$B$82&amp;8</f>
@@ -10253,7 +10264,7 @@
     </row>
     <row r="482" spans="1:3">
       <c r="A482" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B482">
         <f>"dzi"&amp;Calcul!$B$82&amp;10</f>
@@ -10562,7 +10573,7 @@
     </row>
     <row r="513" spans="1:3">
       <c r="A513" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B513">
         <f>"dzi"&amp;Calcul!$B$82&amp;12</f>
@@ -10871,7 +10882,7 @@
     </row>
     <row r="544" spans="1:3">
       <c r="A544" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B544">
         <f>"dzi"&amp;Calcul!$B$82&amp;14</f>
@@ -11180,7 +11191,7 @@
     </row>
     <row r="575" spans="1:3">
       <c r="A575" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B575">
         <f>"dzi"&amp;Calcul!$B$82&amp;16</f>
@@ -11489,7 +11500,7 @@
     </row>
     <row r="606" spans="1:3">
       <c r="A606" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B606">
         <f>"dzi"&amp;Calcul!$B$82&amp;18</f>
@@ -11798,7 +11809,7 @@
     </row>
     <row r="637" spans="1:3">
       <c r="A637" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B637">
         <f>LEFT(MID('Paramètres'!$D$2,MOD(C361,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C361/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C391,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C391/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C421,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C421/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C451,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C451/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C481,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C481/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C512,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C512/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C543,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C543/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C574,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C574/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C605,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C605/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C636,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C636/32),32)+1,1),20)</f>
@@ -11807,12 +11818,12 @@
     </row>
     <row r="639" spans="1:3">
       <c r="A639" s="49" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="640" spans="1:3">
       <c r="A640" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B640">
         <f>"rty"&amp;Calcul!$B$82&amp;0</f>
@@ -12111,7 +12122,7 @@
     </row>
     <row r="670" spans="1:3">
       <c r="A670" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B670">
         <f>"rty"&amp;Calcul!$B$82&amp;2</f>
@@ -12410,7 +12421,7 @@
     </row>
     <row r="700" spans="1:3">
       <c r="A700" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B700">
         <f>"rty"&amp;Calcul!$B$82&amp;4</f>
@@ -12709,7 +12720,7 @@
     </row>
     <row r="730" spans="1:3">
       <c r="A730" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B730">
         <f>"rty"&amp;Calcul!$B$82&amp;6</f>
@@ -13008,7 +13019,7 @@
     </row>
     <row r="760" spans="1:3">
       <c r="A760" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B760">
         <f>"rty"&amp;Calcul!$B$82&amp;8</f>
@@ -13307,7 +13318,7 @@
     </row>
     <row r="790" spans="1:3">
       <c r="A790" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B790">
         <f>LEFT(MID('Paramètres'!$D$2,MOD(C669,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C669/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C699,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C699/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C729,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C729/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C759,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C759/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C789,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C789/32),32)+1,1),10)</f>
@@ -13316,12 +13327,12 @@
     </row>
     <row r="792" spans="1:3">
       <c r="A792" s="49" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="793" spans="1:3">
       <c r="A793" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B793">
         <f>"lve"&amp;Calcul!$B$82&amp;0</f>
@@ -13620,7 +13631,7 @@
     </row>
     <row r="823" spans="1:3">
       <c r="A823" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B823">
         <f>"lve"&amp;Calcul!$B$82&amp;2</f>
@@ -13919,7 +13930,7 @@
     </row>
     <row r="853" spans="1:3">
       <c r="A853" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B853">
         <f>"lve"&amp;Calcul!$B$82&amp;4</f>
@@ -14218,7 +14229,7 @@
     </row>
     <row r="883" spans="1:3">
       <c r="A883" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B883">
         <f>"lve"&amp;Calcul!$B$82&amp;6</f>
@@ -14517,7 +14528,7 @@
     </row>
     <row r="913" spans="1:3">
       <c r="A913" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B913">
         <f>"lve"&amp;Calcul!$B$82&amp;8</f>
@@ -14816,7 +14827,7 @@
     </row>
     <row r="943" spans="1:3">
       <c r="A943" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B943">
         <f>LEFT(MID('Paramètres'!$D$2,MOD(C822,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C822/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C852,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C852/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C882,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C882/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C912,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C912/32),32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(C942,32)+1,1)&amp;MID('Paramètres'!$D$2,MOD(INT(C942/32),32)+1,1),10)</f>
@@ -14825,10 +14836,10 @@
     </row>
     <row r="945" spans="1:5">
       <c r="A945" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B945">
-        <f>IF(ISNUMBER('Racco D2'!$H$29),'Racco D2'!$H$29+'Paramètres'!$B$2,"")</f>
+        <f>IF(ISNUMBER(v_dep),v_dep+'Paramètres'!$B$2,"")</f>
         <v>0</v>
       </c>
       <c r="C945">
@@ -14846,10 +14857,10 @@
     </row>
     <row r="946" spans="1:5">
       <c r="A946" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B946">
-        <f>IF(ISNUMBER('Racco D2'!$H$29),'Racco D2'!$H$29+'Paramètres'!$B$3,"")</f>
+        <f>IF(ISNUMBER(v_dep),v_dep+'Paramètres'!$B$3,"")</f>
         <v>0</v>
       </c>
       <c r="C946">

</xml_diff>